<commit_message>
feat: make Excel spreadsheet generation dynamic, fetch blogs directly from MongoDB, and migrate script to TypeScript
</commit_message>
<xml_diff>
--- a/website_pages_seo_audit.xlsx
+++ b/website_pages_seo_audit.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="177">
   <si>
     <t>SEO Notes / Updates</t>
   </si>
@@ -220,7 +220,127 @@
     <t>Legal policies. Included in sitemap.xml.</t>
   </si>
   <si>
-    <t>WordPress SEO Freelancer</t>
+    <t>How to Start Freelancing as a Student</t>
+  </si>
+  <si>
+    <t>/blog/how-to-start-freelancing-as-a-student</t>
+  </si>
+  <si>
+    <t>https://www.sharikrasool.com/blog/how-to-start-freelancing-as-a-student</t>
+  </si>
+  <si>
+    <t>Learn how to start freelancing as a student, choose profitable skills, build a portfolio, find clients, and gain real-world experience.</t>
+  </si>
+  <si>
+    <t>Live DB Blog Post. Last updated on 6/11/2026.</t>
+  </si>
+  <si>
+    <t>Freelancing vs Entrepreneurship: Which Career Path Is Right for You?</t>
+  </si>
+  <si>
+    <t>/blog/freelancing-vs-entrepreneurship-career-guide</t>
+  </si>
+  <si>
+    <t>https://www.sharikrasool.com/blog/freelancing-vs-entrepreneurship-career-guide</t>
+  </si>
+  <si>
+    <t>Freelancing vs Entrepreneurship: Key Differences &amp; Benefits</t>
+  </si>
+  <si>
+    <t>Explore the differences between freelancing &amp; entrepreneurship. Learn the pros, cons, earning potential, and how to choose the right career path for your goals.</t>
+  </si>
+  <si>
+    <t>Freelance Social Media Manager Tips to Get More Clients</t>
+  </si>
+  <si>
+    <t>/blog/freelance-social-media-manager-tips</t>
+  </si>
+  <si>
+    <t>https://www.sharikrasool.com/blog/freelance-social-media-manager-tips</t>
+  </si>
+  <si>
+    <t>Grow as a Freelance Social Media Manager &amp; Get More Clients</t>
+  </si>
+  <si>
+    <t>Learn freelance social media manager tips to get more clients, improve your online presence, and grow your freelancing career successfully.</t>
+  </si>
+  <si>
+    <t>How to Write a Freelancing Resume That Attracts Clients and Remote Jobs</t>
+  </si>
+  <si>
+    <t>/blog/how-to-write-a-freelancing-resume</t>
+  </si>
+  <si>
+    <t>https://www.sharikrasool.com/blog/how-to-write-a-freelancing-resume</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Freelancing Resume Tips to Win Clients and Remote Jobs</t>
+  </si>
+  <si>
+    <t>Learn how to create a professional freelancing resume that attracts clients, boosts credibility, and helps secure remote jobs.</t>
+  </si>
+  <si>
+    <t>Best Freelancing Ideas to Build a Successful Career Online</t>
+  </si>
+  <si>
+    <t>/blog/best-freelancing-ideas-to-build-career</t>
+  </si>
+  <si>
+    <t>https://www.sharikrasool.com/blog/best-freelancing-ideas-to-build-career</t>
+  </si>
+  <si>
+    <t>Smart Freelancing Ideas to Succeed in the Online World.</t>
+  </si>
+  <si>
+    <t>Explore the best freelancing ideas including SEO, web development and AI services. Build a profitable and scalable online freelance career today.</t>
+  </si>
+  <si>
+    <t>Understanding the Pros and Cons of Freelancing in Today’s Job Market</t>
+  </si>
+  <si>
+    <t>/blog/the-pros-and-cons-of-freelancing</t>
+  </si>
+  <si>
+    <t>https://www.sharikrasool.com/blog/the-pros-and-cons-of-freelancing</t>
+  </si>
+  <si>
+    <t>Pros and Cons of Freelancing: Benefits, Risks &amp; Career Insights</t>
+  </si>
+  <si>
+    <t>Explore the pros and cons of freelancing, including benefits, challenges, income stability, and career growth to decide if freelancing is right for you</t>
+  </si>
+  <si>
+    <t>Freelancing Tips That Actually Work: How to Build a Stable, High-Income Freelance Career</t>
+  </si>
+  <si>
+    <t>/blog/freelancing-tips-that-actually-works</t>
+  </si>
+  <si>
+    <t>https://www.sharikrasool.com/blog/freelancing-tips-that-actually-works</t>
+  </si>
+  <si>
+    <t>Freelancing Tips to Build a Successful Career</t>
+  </si>
+  <si>
+    <t>Discover proven freelancing tips to get clients, price your services, and build a stable, profitable freelance career step by step.</t>
+  </si>
+  <si>
+    <t>How to Start Freelancing With No Experience (Beginner’s Guide)</t>
+  </si>
+  <si>
+    <t>/blog/how-to-start-freelancing-for-beginners</t>
+  </si>
+  <si>
+    <t>https://www.sharikrasool.com/blog/how-to-start-freelancing-for-beginners</t>
+  </si>
+  <si>
+    <t>How to Start Freelancing From Scratch (Beginner Roadmap)</t>
+  </si>
+  <si>
+    <t>Confused about freelancing? This beginner guide shows how to start freelancing, build a portfolio, find clients, and grow income step by step.</t>
+  </si>
+  <si>
+    <t>WordPress SEO Freelancer: Who They Are, Benefits, Services &amp; Hiring Guide</t>
   </si>
   <si>
     <t>/blog/wordpress-seo-freelancer</t>
@@ -229,133 +349,10 @@
     <t>https://www.sharikrasool.com/blog/wordpress-seo-freelancer</t>
   </si>
   <si>
-    <t>WordPress SEO Freelancer | SaaS Search Rankings growth</t>
-  </si>
-  <si>
-    <t>Hire a professional WordPress SEO freelancer to optimize content hierarchy, crawl efficiency, meta tags, and build clean internal backlinks.</t>
-  </si>
-  <si>
-    <t>CMS published post. Repetitive brand suffix cleaned.</t>
-  </si>
-  <si>
-    <t>How to Start Freelancing for Beginners</t>
-  </si>
-  <si>
-    <t>/blog/how-to-start-freelancing-for-beginners</t>
-  </si>
-  <si>
-    <t>https://www.sharikrasool.com/blog/how-to-start-freelancing-for-beginners</t>
-  </si>
-  <si>
-    <t>How to Start Freelancing for Beginners | Step-by-Step Guide</t>
-  </si>
-  <si>
-    <t>A complete starter guide to choosing a niche, setting up your freelance services, and landing your first client with zero experience.</t>
-  </si>
-  <si>
-    <t>9 Freelancing Tips That Actually Work</t>
-  </si>
-  <si>
-    <t>/blog/freelancing-tips-that-actually-works</t>
-  </si>
-  <si>
-    <t>https://www.sharikrasool.com/blog/freelancing-tips-that-actually-works</t>
-  </si>
-  <si>
-    <t>9 Freelancing Tips That Actually Work | Scale Your Business</t>
-  </si>
-  <si>
-    <t>Actionable freelancing tips and productivity strategies for growing client contracts, structuring fees, and managing work-life balance.</t>
-  </si>
-  <si>
-    <t>The Pros and Cons of Freelancing</t>
-  </si>
-  <si>
-    <t>/blog/the-pros-and-cons-of-freelancing</t>
-  </si>
-  <si>
-    <t>https://www.sharikrasool.com/blog/the-pros-and-cons-of-freelancing</t>
-  </si>
-  <si>
-    <t>The Pros and Cons of Freelancing | Career Choice Breakdown</t>
-  </si>
-  <si>
-    <t>We weigh the advantages of flexible work schedules and freedom against the disadvantages of client acquisition and unstable income.</t>
-  </si>
-  <si>
-    <t>15 Best Freelancing Ideas to Build Career</t>
-  </si>
-  <si>
-    <t>/blog/best-freelancing-ideas-to-build-career</t>
-  </si>
-  <si>
-    <t>https://www.sharikrasool.com/blog/best-freelancing-ideas-to-build-career</t>
-  </si>
-  <si>
-    <t>15 Best Freelancing Ideas to Build a Profitable Career</t>
-  </si>
-  <si>
-    <t>Explore high-demand freelance career fields, including coding, SEO, copywriting, and design, to kickstart your freelancing journey.</t>
-  </si>
-  <si>
-    <t>How to Write a Freelance Resume</t>
-  </si>
-  <si>
-    <t>/blog/how-to-write-a-freelancing-resume</t>
-  </si>
-  <si>
-    <t>https://www.sharikrasool.com/blog/how-to-write-a-freelancing-resume</t>
-  </si>
-  <si>
-    <t>How to Write a Freelance Resume | Portfolios and Formats</t>
-  </si>
-  <si>
-    <t>Learn how to structure a professional freelance resume to showcase contract projects, portfolios, and key skills to land corporate gigs.</t>
-  </si>
-  <si>
-    <t>Freelance Social Media Manager Tips</t>
-  </si>
-  <si>
-    <t>/blog/freelance-social-media-manager-tips</t>
-  </si>
-  <si>
-    <t>https://www.sharikrasool.com/blog/freelance-social-media-manager-tips</t>
-  </si>
-  <si>
-    <t>Freelance Social Media Manager Tips | Client Acquisition</t>
-  </si>
-  <si>
-    <t>Expert tips for freelance social media managers on onboarding clients, scaling content plans, and tracking engagement metrics.</t>
-  </si>
-  <si>
-    <t>Freelancing vs Entrepreneurship Career Guide</t>
-  </si>
-  <si>
-    <t>/blog/freelancing-vs-entrepreneurship-career-guide</t>
-  </si>
-  <si>
-    <t>https://www.sharikrasool.com/blog/freelancing-vs-entrepreneurship-career-guide</t>
-  </si>
-  <si>
-    <t>Freelancing vs Entrepreneurship | Which Career is Best?</t>
-  </si>
-  <si>
-    <t>An in-depth comparison of freelance service contracts versus building a scalable startup business to find your perfect career path.</t>
-  </si>
-  <si>
-    <t>How to Start Freelancing as a Student</t>
-  </si>
-  <si>
-    <t>/blog/how-to-start-freelancing-as-a-student</t>
-  </si>
-  <si>
-    <t>https://www.sharikrasool.com/blog/how-to-start-freelancing-as-a-student</t>
-  </si>
-  <si>
-    <t>How to Start Freelancing as a Student | Earn While Studying</t>
-  </si>
-  <si>
-    <t>Learn how to balance university classes while earning a freelance income online with easy high-income digital service niches.</t>
+    <t>WordPress SEO Freelancer: Services &amp; Hiring Guide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A walk through who a WordPress SEO freelancer is, what they do, the benefits they bring, and how to choose the right one for your business. </t>
   </si>
   <si>
     <t>AI Image Prompt Generator</t>
@@ -565,7 +562,7 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="16"/>
+      <sz val="14"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -1489,10 +1486,10 @@
         <v>70</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>71</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>72</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>15</v>
@@ -1507,30 +1504,30 @@
         <v>18</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>78</v>
-      </c>
       <c r="F6" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>17</v>
@@ -1539,30 +1536,30 @@
         <v>18</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>83</v>
-      </c>
       <c r="F7" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>17</v>
@@ -1571,30 +1568,30 @@
         <v>18</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>88</v>
-      </c>
       <c r="F8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>17</v>
@@ -1603,30 +1600,30 @@
         <v>18</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="F9" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>17</v>
@@ -1635,30 +1632,30 @@
         <v>18</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>98</v>
-      </c>
       <c r="F10" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>17</v>
@@ -1667,30 +1664,30 @@
         <v>18</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>103</v>
-      </c>
       <c r="F11" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>17</v>
@@ -1699,30 +1696,30 @@
         <v>18</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>108</v>
-      </c>
       <c r="F12" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>17</v>
@@ -1731,30 +1728,30 @@
         <v>18</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>113</v>
-      </c>
       <c r="F13" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>17</v>
@@ -1763,7 +1760,7 @@
         <v>18</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1863,57 +1860,57 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>124</v>
-      </c>
       <c r="F6" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>17</v>
@@ -1922,30 +1919,30 @@
         <v>18</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>129</v>
-      </c>
       <c r="F7" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>17</v>
@@ -1954,30 +1951,30 @@
         <v>18</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="E8" s="5" t="s">
-        <v>134</v>
-      </c>
       <c r="F8" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>17</v>
@@ -1986,30 +1983,30 @@
         <v>18</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>139</v>
-      </c>
       <c r="F9" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>17</v>
@@ -2018,30 +2015,30 @@
         <v>18</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>144</v>
-      </c>
       <c r="F10" s="5" t="s">
         <v>15</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>17</v>
@@ -2050,30 +2047,30 @@
         <v>18</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="D11" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>149</v>
-      </c>
       <c r="F11" s="3" t="s">
         <v>15</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>17</v>
@@ -2082,7 +2079,7 @@
         <v>18</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -2182,194 +2179,194 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>160</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>164</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J8" s="5" t="s">
         <v>168</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" s="3" t="s">
         <v>172</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="5" t="s">
         <v>176</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>